<commit_message>
feat: add customizable packaging units, optimize mobile card UI, and improve AI billing assistant
</commit_message>
<xml_diff>
--- a/sample_invoice_template.xlsx
+++ b/sample_invoice_template.xlsx
@@ -997,67 +997,103 @@
       <c r="I22" s="22" t="n"/>
     </row>
     <row r="23" ht="16.8" customHeight="1">
-      <c r="A23" s="5" t="n"/>
-      <c r="F23" s="23" t="n"/>
-      <c r="G23" s="24" t="n"/>
-      <c r="H23" s="25" t="n"/>
+      <c r="A23" s="18" t="n"/>
+      <c r="B23" s="11" t="n"/>
+      <c r="C23" s="11" t="n"/>
+      <c r="D23" s="11" t="n"/>
+      <c r="E23" s="11" t="n"/>
+      <c r="F23" s="19" t="n"/>
+      <c r="G23" s="20" t="n"/>
+      <c r="H23" s="21" t="n"/>
       <c r="I23" s="22" t="n"/>
     </row>
     <row r="24" ht="16.8" customHeight="1">
-      <c r="A24" s="5" t="n"/>
-      <c r="F24" s="26" t="n"/>
-      <c r="G24" s="26" t="n"/>
-      <c r="H24" s="26" t="n"/>
-      <c r="I24" s="7" t="n"/>
+      <c r="A24" s="18" t="n"/>
+      <c r="B24" s="11" t="n"/>
+      <c r="C24" s="11" t="n"/>
+      <c r="D24" s="11" t="n"/>
+      <c r="E24" s="11" t="n"/>
+      <c r="F24" s="19" t="n"/>
+      <c r="G24" s="20" t="n"/>
+      <c r="H24" s="21" t="n"/>
+      <c r="I24" s="22" t="n"/>
     </row>
     <row r="25" ht="16.8" customHeight="1">
-      <c r="A25" s="5" t="n"/>
-      <c r="F25" s="26" t="n"/>
-      <c r="G25" s="26" t="n"/>
-      <c r="H25" s="26" t="n"/>
-      <c r="I25" s="7" t="n"/>
+      <c r="A25" s="18" t="n"/>
+      <c r="B25" s="11" t="n"/>
+      <c r="C25" s="11" t="n"/>
+      <c r="D25" s="11" t="n"/>
+      <c r="E25" s="11" t="n"/>
+      <c r="F25" s="19" t="n"/>
+      <c r="G25" s="20" t="n"/>
+      <c r="H25" s="21" t="n"/>
+      <c r="I25" s="22" t="n"/>
     </row>
     <row r="26" ht="16.8" customHeight="1">
-      <c r="A26" s="5" t="n"/>
-      <c r="F26" s="26" t="n"/>
-      <c r="G26" s="26" t="n"/>
-      <c r="H26" s="26" t="n"/>
-      <c r="I26" s="7" t="n"/>
+      <c r="A26" s="18" t="n"/>
+      <c r="B26" s="11" t="n"/>
+      <c r="C26" s="11" t="n"/>
+      <c r="D26" s="11" t="n"/>
+      <c r="E26" s="11" t="n"/>
+      <c r="F26" s="19" t="n"/>
+      <c r="G26" s="20" t="n"/>
+      <c r="H26" s="21" t="n"/>
+      <c r="I26" s="22" t="n"/>
     </row>
     <row r="27" ht="16.8" customHeight="1">
-      <c r="A27" s="5" t="n"/>
-      <c r="F27" s="26" t="n"/>
-      <c r="G27" s="26" t="n"/>
-      <c r="H27" s="26" t="n"/>
-      <c r="I27" s="7" t="n"/>
+      <c r="A27" s="18" t="n"/>
+      <c r="B27" s="11" t="n"/>
+      <c r="C27" s="11" t="n"/>
+      <c r="D27" s="11" t="n"/>
+      <c r="E27" s="11" t="n"/>
+      <c r="F27" s="19" t="n"/>
+      <c r="G27" s="20" t="n"/>
+      <c r="H27" s="21" t="n"/>
+      <c r="I27" s="22" t="n"/>
     </row>
     <row r="28" ht="16.8" customHeight="1">
-      <c r="A28" s="5" t="n"/>
-      <c r="F28" s="26" t="n"/>
-      <c r="G28" s="26" t="n"/>
-      <c r="H28" s="26" t="n"/>
-      <c r="I28" s="7" t="n"/>
+      <c r="A28" s="18" t="n"/>
+      <c r="B28" s="11" t="n"/>
+      <c r="C28" s="11" t="n"/>
+      <c r="D28" s="11" t="n"/>
+      <c r="E28" s="11" t="n"/>
+      <c r="F28" s="19" t="n"/>
+      <c r="G28" s="20" t="n"/>
+      <c r="H28" s="21" t="n"/>
+      <c r="I28" s="22" t="n"/>
     </row>
     <row r="29" ht="16.8" customHeight="1">
-      <c r="A29" s="5" t="n"/>
-      <c r="F29" s="26" t="n"/>
-      <c r="G29" s="26" t="n"/>
-      <c r="H29" s="26" t="n"/>
-      <c r="I29" s="7" t="n"/>
+      <c r="A29" s="18" t="n"/>
+      <c r="B29" s="11" t="n"/>
+      <c r="C29" s="11" t="n"/>
+      <c r="D29" s="11" t="n"/>
+      <c r="E29" s="11" t="n"/>
+      <c r="F29" s="19" t="n"/>
+      <c r="G29" s="20" t="n"/>
+      <c r="H29" s="21" t="n"/>
+      <c r="I29" s="22" t="n"/>
     </row>
     <row r="30" ht="12" customHeight="1">
-      <c r="A30" s="5" t="n"/>
-      <c r="F30" s="26" t="n"/>
-      <c r="G30" s="26" t="n"/>
-      <c r="H30" s="26" t="n"/>
-      <c r="I30" s="7" t="n"/>
+      <c r="A30" s="18" t="n"/>
+      <c r="B30" s="11" t="n"/>
+      <c r="C30" s="11" t="n"/>
+      <c r="D30" s="11" t="n"/>
+      <c r="E30" s="11" t="n"/>
+      <c r="F30" s="19" t="n"/>
+      <c r="G30" s="20" t="n"/>
+      <c r="H30" s="21" t="n"/>
+      <c r="I30" s="22" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="5" t="n"/>
-      <c r="F31" s="26" t="n"/>
-      <c r="G31" s="26" t="n"/>
-      <c r="H31" s="26" t="n"/>
-      <c r="I31" s="47" t="n"/>
+      <c r="A31" s="18" t="n"/>
+      <c r="B31" s="11" t="n"/>
+      <c r="C31" s="11" t="n"/>
+      <c r="D31" s="11" t="n"/>
+      <c r="E31" s="11" t="n"/>
+      <c r="F31" s="19" t="n"/>
+      <c r="G31" s="20" t="n"/>
+      <c r="H31" s="21" t="n"/>
+      <c r="I31" s="22" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="5" t="n"/>

</xml_diff>